<commit_message>
Add detailed Class 4 cost estimate sheet (AACE 18R-97, 5-15% design maturity)
New 'Class 4 Estimate' sheet with WBS-level breakdown:
- WBS 1.0: SSA RF Source (modules, spares, design study, test stand)
- WBS 2.0: RF Distribution (combiners, waveguide, circulators, loads)
- WBS 3.0: Control Electronics (LLRF9, Interface Chassis, MPS, arc detect, waveform buffer, tuners, PPS)
- WBS 4.0: Software (EPICS IOC, state machine, operator panels, commissioning tools)
- WBS 5.0: Installation and Commissioning (per-station phased turn-on)
- WBS 6.0: Site Prep (waveguide removal, cable tray, equipment relocation)
- WBS 7.0: Project Management (PM, safety reviews)
- WBS 8.0: Infrastructure Reference (electrical, water, building - other groups)

Each line item includes M&S, labor FTE, basis of estimate with source references,
and confidence level (H/M/L). Key assumptions and risks documented.

Co-authored-by: fayaw <faya.wang@gmail.com>
</commit_message>
<xml_diff>
--- a/SSA_upgrade/SSA Upgrade Project Cost V1.xlsx
+++ b/SSA_upgrade/SSA Upgrade Project Cost V1.xlsx
@@ -6,8 +6,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="8460" yWindow="5385" windowWidth="20955" windowHeight="16425" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cover page" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SSA quote from R&amp;K" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Class 4 Estimate" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cover page" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SSA quote from R&amp;K" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -16,8 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="4">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.0"/>
+  </numFmts>
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,16 +40,76 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E2F3"/>
+        <bgColor rgb="00D9E2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6B8B7"/>
+        <bgColor rgb="00E6B8B7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -69,11 +132,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="2"/>
@@ -87,6 +156,19 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -430,6 +512,1877 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H84"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>SPEAR3 SSA Upgrade Project - Class 4 Cost Estimate (AACE 18R-97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Design Maturity: 5-15%  |  Labor Rate: $200/hr burdened  |  1 FTE = 1,740 hrs/yr  |  All costs in k$  |  Base year: 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>WBS</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>M&amp;S (k$)</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Labor (FTE)</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Labor (k$)</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Total (k$)</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>Conf.</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>Basis of Estimate / Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>SSA RF SOURCE</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n"/>
+      <c r="D6" s="10" t="n"/>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="10" t="n"/>
+      <c r="H6" s="10" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>SSA Modules (16 x 65 kW, R&amp;K Company)</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>4985.6</v>
+      </c>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n">
+        <v>4985.6</v>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>R&amp;K quote July 2025: $311,600/unit x 16 = $4,985,600. 476.3 MHz CW. Includes internal PS, LCW cooling, VSWR protection, Ethernet/serial control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>SSA Spare Modules (2 units)</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>623.2</v>
+      </c>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n">
+        <v>623.2</v>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>2 hot-swap spares @ $311,600 each. Industry practice for 16-module system. Enables rapid module replacement without waiting for vendor lead time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>SSA Design Study &amp; Prototype Test</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>348</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>348</v>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>0.5 FTE prototype design + 0.5 FTE vendor collaboration and test iteration. Includes acceptance test protocol development. Per cover page row 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>SSA Test Stand (Bldg 122)</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>75</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>174</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>249</v>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>High-power RF load (50 kW CW), power measurement, 480V service, LCW (~15 GPM per 3/10 mtg). Existing Bldg 122 LCW connection usable. 0.5 FTE setup/integration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr"/>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Subtotal WBS 1.0</t>
+        </is>
+      </c>
+      <c r="C11" s="12">
+        <f>SUM(C7:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="12" t="n"/>
+      <c r="E11" s="12">
+        <f>SUM(E7:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="12">
+        <f>SUM(F7:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="12" t="n"/>
+      <c r="H11" s="12" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>RF DISTRIBUTION &amp; COMBINING</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
+      <c r="H13" s="10" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>6-1/8" Coaxial Combiners (4 x 4:1)</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>160</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>87</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>247</v>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>4 combiners, each combining 4 SSA outputs (6-1/8" coax) into single WR2100 port. ~$40k each installed. Each SSA cabinet outputs 6-1/8" coax per 3/10 mtg notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>WR2100 Waveguide Runs (4 independent)</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>300</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>174</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>474</v>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>4 independent WR2100 runs from SSA bldg to 4 cavities. Straight sections, H/E-plane bends, flex sections. ~10 lb/ft, Unistrut hangers every 8 ft. Lambda_g=80.4 cm at 476.3 MHz; lengths matched to +/- n*lambda_g.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Circulators (4 x 250+ kW @ 476 MHz)</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>400</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>452.2</v>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t>4 ferrite circulators, one per combined output. $80-120k each NEW. NOTE: PEP-II 1.5 MW circulators available (per 2/24 mtg) - if reusable, M&amp;S drops to ~$0. Carry new-buy as baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>RF Loads (circulator loads, terminations)</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>80</v>
+      </c>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n">
+        <v>80</v>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H17" s="11" t="inlineStr">
+        <is>
+          <t>4 circulator loads (water-cooled, ~250 kW each), waveguide terminations, dummy loads for commissioning. Loads cooled by HCW (separate from LCW per 3/10 mtg).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Directional Couplers &amp; Transitions</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t>Directional couplers at each combined output (4) and at each SSA output (16 may be internal). WR2100-to-coax transitions. Phase trimmers for combining efficiency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Waveguide Supports, Hangers, Hardware</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>87</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>137</v>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t>Unistrut channel, beam clamps, waveguide hangers every 8 ft, mounting hardware. Some supports from equipment platform structure above (per 3/10 mtg).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr"/>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Subtotal WBS 2.0</t>
+        </is>
+      </c>
+      <c r="C20" s="12">
+        <f>SUM(C14:C19)</f>
+        <v/>
+      </c>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="12">
+        <f>SUM(E14:E19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="12">
+        <f>SUM(F14:F19)</f>
+        <v/>
+      </c>
+      <c r="G20" s="12" t="n"/>
+      <c r="H20" s="12" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>CONTROL ELECTRONICS</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="10" t="n"/>
+      <c r="H22" s="10" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>LLRF9 Controllers (4 x Dimtel LLRF9/500)</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>398</v>
+      </c>
+      <c r="D23" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E23" s="11" t="n">
+        <v>174</v>
+      </c>
+      <c r="F23" s="11" t="n">
+        <v>572</v>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="H23" s="11" t="inlineStr">
+        <is>
+          <t>Dimtel LLRF9/500 list $117k; 15% vol discount = $99.45k each x 4 = $397.8k. Each unit: 9 RF channels, FPGA interlocks &lt;1us, built-in EPICS IOC, 10 Hz scalar readback. 0.5 FTE for integration/configuration. Per LLRFUpgradeTaskListRev3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Interface Chassis (SSA topology)</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D24" s="11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>261</v>
+      </c>
+      <c r="F24" s="11" t="n">
+        <v>286</v>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>Central interlock hub: AND-logic, first-fault latching, fiber-optic HVPS ctrl, &lt;1us response. SSA version needs per-station permit logic + module-level status. PCB design + fabrication + chassis. CRITICAL PATH per 0_SYSTEM_DESIGN_REPORT.md Sec 8.3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>RF MPS PLC (ControlLogix 1756)</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D25" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E25" s="11" t="n">
+        <v>174</v>
+      </c>
+      <c r="F25" s="11" t="n">
+        <v>204</v>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="H25" s="11" t="inlineStr">
+        <is>
+          <t>AB ControlLogix PLC: $22k/set (detailed BOM in TaskListRev3: 5069-L320ER $3.7k, OF8 $1.5k x3, OX41 $451 x10, etc). SSA needs expanded I/O for 16 modules. +$8k for additional I/O modules. 0.5 FTE PLC programming + EPICS IOC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Arc Detection System</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D26" s="11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E26" s="11" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="F26" s="11" t="n">
+        <v>124.4</v>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="H26" s="11" t="inlineStr">
+        <is>
+          <t>Microstep-MIS sensors 470EUR x10=$5.1k, receivers 635EUR x6=$4.1k, cables=$1.1k, DB25=$200, mech adapters=$7k. Per TaskListRev3 quote from Erik Bystricky Nov 2024. 10 sensors (8 cavity + 1 kly + 1 circ), 5+1 receivers. Arc Detection Chassis: OR-gate + 10-bit latch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Waveform Buffer System</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D27" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>174</v>
+      </c>
+      <c r="F27" s="11" t="n">
+        <v>189</v>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H27" s="11" t="inlineStr">
+        <is>
+          <t>Custom chassis: 8 RF + 4 HVPS channels, circular buffers, analog comparator trips, enhanced collector power protection algorithm. MCL ZX47-40LN-S+ detectors ($1.7k) + signal conditioning opamps + ADCs + chassis. Per WaveformBuffersforLLRFUpgrade.docx (Sebek, Jan 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>SSA Module Status Monitoring</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D28" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E28" s="11" t="n">
+        <v>87</v>
+      </c>
+      <c r="F28" s="11" t="n">
+        <v>102</v>
+      </c>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="inlineStr">
+        <is>
+          <t>Per-module monitoring: VSWR, output power, temperature, fault status x16 modules. Ethernet/serial polling + analog readback. May be integrated into MPS PLC I/O or dedicated monitoring chassis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Tuner Motor Controllers (4 x Galil DMC-4143)</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D29" s="11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E29" s="11" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="F29" s="11" t="n">
+        <v>114.4</v>
+      </c>
+      <c r="G29" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H29" s="11" t="inlineStr">
+        <is>
+          <t>Galil DMC-4143 4-axis controller $1,675 each x2 (1 operational + 1 spare). Motor drivers, cables, encoder interfaces. EPICS motor record support. Per galil/ commissioning docs. RISK: reliability TBD - test on booster tuners first (Sec 10.6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>3.8</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>PPS Interface Box</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D30" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E30" s="11" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="F30" s="11" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="H30" s="11" t="inlineStr">
+        <is>
+          <t>Small Bud enclosure ~6x5x4in, 4 relays, status LEDs, inhibit buttons. Proven design per Ben Morris 3/5/2026 (pps_Ben.md). Identical to gallery/6575 modulator systems. Requires PPS group review and RSWCF. $2-5k materials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Cables, Connectors, Integration Materials</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H31" s="11" t="inlineStr">
+        <is>
+          <t>RF cables (SMA, Type-N), fiber optic links (HFBR-1412/2412), LEMO interlock cables, multi-conductor digital cables, power supplies, rack hardware, PDUs, labels. ~10% of WBS 3.1-3.8 hardware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr"/>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>Subtotal WBS 3.0</t>
+        </is>
+      </c>
+      <c r="C32" s="12">
+        <f>SUM(C23:C31)</f>
+        <v/>
+      </c>
+      <c r="D32" s="12" t="n"/>
+      <c r="E32" s="12">
+        <f>SUM(E23:E31)</f>
+        <v/>
+      </c>
+      <c r="F32" s="12">
+        <f>SUM(F23:F31)</f>
+        <v/>
+      </c>
+      <c r="G32" s="12" t="n"/>
+      <c r="H32" s="12" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>SOFTWARE &amp; INTEGRATION</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="n"/>
+      <c r="D34" s="10" t="n"/>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="10" t="n"/>
+      <c r="G34" s="10" t="n"/>
+      <c r="H34" s="10" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>EPICS IOC Development</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D35" s="11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E35" s="11" t="n">
+        <v>261</v>
+      </c>
+      <c r="F35" s="11" t="n">
+        <v>271</v>
+      </c>
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H35" s="11" t="inlineStr">
+        <is>
+          <t>IOCs for: LLRF9 (Dimtel provides baseline, SPEAR customization), MPS ControlLogix (EtherIP/pycomm3), SSA module monitoring (ASYN/StreamDevice), Waveform Buffer, Chroma heater ASYN driver. Dev tools + test licenses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>State Machine / EPICS Coordinator</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="n"/>
+      <c r="D36" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="11" t="n">
+        <v>348</v>
+      </c>
+      <c r="F36" s="11" t="n">
+        <v>348</v>
+      </c>
+      <c r="G36" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H36" s="11" t="inlineStr">
+        <is>
+          <t>Python/MATLAB supervisory control ~1 Hz. States: OFF/PARK/TUNE/ON_CW. Fault handling, auto-recovery, HVPS ramp control, heater warm-up/cooldown sequences. Load angle offset loop (balance 4 cavity fields). CRITICAL: largest untouched software scope per Sec 19.3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Operator Interface (EDM/CSS Panels)</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="n"/>
+      <c r="D37" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E37" s="11" t="n">
+        <v>87</v>
+      </c>
+      <c r="F37" s="11" t="n">
+        <v>87</v>
+      </c>
+      <c r="G37" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H37" s="11" t="inlineStr">
+        <is>
+          <t>EDM/CSS operator displays: station overview, per-module SSA status, LLRF9 summary, MPS fault tree, waveform displays, tuner positions, HVPS status. Based on existing rf_station_4CVSPR.edl pattern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Commissioning Tools &amp; Scripts</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D38" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E38" s="11" t="n">
+        <v>87</v>
+      </c>
+      <c r="F38" s="11" t="n">
+        <v>92</v>
+      </c>
+      <c r="G38" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H38" s="11" t="inlineStr">
+        <is>
+          <t>MATLAB/Python tools for: SSA phase calibration, combiner efficiency optimization, interlock chain verification, automated fault injection testing, performance logging. Per legacy rf_calib.st (2,800+ lines).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Documentation &amp; Training</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E39" s="11" t="n">
+        <v>87</v>
+      </c>
+      <c r="F39" s="11" t="n">
+        <v>87</v>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H39" s="11" t="inlineStr">
+        <is>
+          <t>System documentation, as-built drawings, operator training materials, maintenance procedures. ~25 schematics for MPS + ~25 for HVPS (per TaskListRev3). Training for operations staff on new SSA system.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr"/>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>Subtotal WBS 4.0</t>
+        </is>
+      </c>
+      <c r="C40" s="12">
+        <f>SUM(C35:C39)</f>
+        <v/>
+      </c>
+      <c r="D40" s="12" t="n"/>
+      <c r="E40" s="12">
+        <f>SUM(E35:E39)</f>
+        <v/>
+      </c>
+      <c r="F40" s="12">
+        <f>SUM(F35:F39)</f>
+        <v/>
+      </c>
+      <c r="G40" s="12" t="n"/>
+      <c r="H40" s="12" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>INSTALLATION &amp; COMMISSIONING</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="n"/>
+      <c r="D42" s="10" t="n"/>
+      <c r="E42" s="10" t="n"/>
+      <c r="F42" s="10" t="n"/>
+      <c r="G42" s="10" t="n"/>
+      <c r="H42" s="10" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>SSA Module Installation (4 stations)</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D43" s="11" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="E43" s="11" t="n">
+        <v>480</v>
+      </c>
+      <c r="F43" s="11" t="n">
+        <v>530</v>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H43" s="11" t="inlineStr">
+        <is>
+          <t>4 person-3 weeks/station x 4 stations = 12 person-months. Rack mounting, 480V power connections, LCW plumbing to each module, RF output cabling, control/interlock wiring. $50k for tools, rigging, consumables. Per cover page row 8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>RF Distribution Installation</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D44" s="11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E44" s="11" t="n">
+        <v>261</v>
+      </c>
+      <c r="F44" s="11" t="n">
+        <v>291</v>
+      </c>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H44" s="11" t="inlineStr">
+        <is>
+          <t>Waveguide assembly, circulator installation (vertical orientation per 2/24 mtg), combiner hookup, load installation. Requires crane for heavy components. Waveguide alignment and RF leak testing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>Controls &amp; Cabling Installation</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D45" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E45" s="11" t="n">
+        <v>174</v>
+      </c>
+      <c r="F45" s="11" t="n">
+        <v>194</v>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H45" s="11" t="inlineStr">
+        <is>
+          <t>LLRF9 rack mounting, MPS PLC wiring, Interface Chassis installation, arc detector fiber routing, interlock cabling, Ethernet network, fiber-optic links to HVPS (HFBR-1412/2412).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>5.4</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>System Integration Testing</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="n"/>
+      <c r="D46" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E46" s="11" t="n">
+        <v>174</v>
+      </c>
+      <c r="F46" s="11" t="n">
+        <v>174</v>
+      </c>
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H46" s="11" t="inlineStr">
+        <is>
+          <t>End-to-end interlock chain testing (Layer 1-4), EPICS PV verification, fault injection testing, waveform capture validation. Limited window due to SPEAR operations (per Sec 19.1 constraint).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>Phased Commissioning (per-station turn-on)</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D47" s="11" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E47" s="11" t="n">
+        <v>240</v>
+      </c>
+      <c r="F47" s="11" t="n">
+        <v>260</v>
+      </c>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H47" s="11" t="inlineStr">
+        <is>
+          <t>6 person-2 months commissioning (per cover page row 8). Incremental power ramp per station. Performance validation: amplitude stability &lt;0.1%, phase &lt;0.1 deg. Includes Dimtel 1-week on-site support per LLRF9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr"/>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>Subtotal WBS 5.0</t>
+        </is>
+      </c>
+      <c r="C48" s="12">
+        <f>SUM(C43:C47)</f>
+        <v/>
+      </c>
+      <c r="D48" s="12" t="n"/>
+      <c r="E48" s="12">
+        <f>SUM(E43:E47)</f>
+        <v/>
+      </c>
+      <c r="F48" s="12">
+        <f>SUM(F43:F47)</f>
+        <v/>
+      </c>
+      <c r="G48" s="12" t="n"/>
+      <c r="H48" s="12" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>SITE PREPARATION &amp; REMOVAL</t>
+        </is>
+      </c>
+      <c r="C50" s="10" t="n"/>
+      <c r="D50" s="10" t="n"/>
+      <c r="E50" s="10" t="n"/>
+      <c r="F50" s="10" t="n"/>
+      <c r="G50" s="10" t="n"/>
+      <c r="H50" s="10" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>Existing Waveguide Removal</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D51" s="11" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E51" s="11" t="n">
+        <v>41.8</v>
+      </c>
+      <c r="F51" s="11" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="H51" s="11" t="inlineStr">
+        <is>
+          <t>Remove existing klystron waveguide (magic tee splitters, existing WR2100 run). Roof waveguide splitters removed; direct 1:1 SSA-to-cavity runs replace them (per 2/24 mtg).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>Cable Tray Relocation</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D52" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E52" s="11" t="n">
+        <v>87</v>
+      </c>
+      <c r="F52" s="11" t="n">
+        <v>97</v>
+      </c>
+      <c r="G52" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H52" s="11" t="inlineStr">
+        <is>
+          <t>Straighten S-shaped cable trays for 4 waveguide runs on roof (per 2/24 mtg). Relocate cable trays between 118 and ring ~10 ft outward for clearance. 4 person-1 month per cover page row 9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="11" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="B53" s="11" t="inlineStr">
+        <is>
+          <t>Equipment Relocation</t>
+        </is>
+      </c>
+      <c r="C53" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D53" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E53" s="11" t="n">
+        <v>87</v>
+      </c>
+      <c r="F53" s="11" t="n">
+        <v>102</v>
+      </c>
+      <c r="G53" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H53" s="11" t="inlineStr">
+        <is>
+          <t>Relocate transformers (2-3), distribution panels, MPS controls cabinets during downtime. Remove old air-handler/chiller behind 507 (per 2/24 mtg). Relocate condensing unit 5-10 ft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="12" t="inlineStr"/>
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>Subtotal WBS 6.0</t>
+        </is>
+      </c>
+      <c r="C54" s="12">
+        <f>SUM(C51:C53)</f>
+        <v/>
+      </c>
+      <c r="D54" s="12" t="n"/>
+      <c r="E54" s="12">
+        <f>SUM(E51:E53)</f>
+        <v/>
+      </c>
+      <c r="F54" s="12">
+        <f>SUM(F51:F53)</f>
+        <v/>
+      </c>
+      <c r="G54" s="12" t="n"/>
+      <c r="H54" s="12" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>PROJECT MANAGEMENT</t>
+        </is>
+      </c>
+      <c r="C56" s="10" t="n"/>
+      <c r="D56" s="10" t="n"/>
+      <c r="E56" s="10" t="n"/>
+      <c r="F56" s="10" t="n"/>
+      <c r="G56" s="10" t="n"/>
+      <c r="H56" s="10" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>Technical Program Management</t>
+        </is>
+      </c>
+      <c r="C57" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D57" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E57" s="11" t="n">
+        <v>870</v>
+      </c>
+      <c r="F57" s="11" t="n">
+        <v>890</v>
+      </c>
+      <c r="G57" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H57" s="11" t="inlineStr">
+        <is>
+          <t>~0.5 FTE/yr average over ~5-year project. Schedule management, resource coordination, vendor management (R&amp;K, Dimtel), progress reporting. M&amp;S for travel to vendor sites, DOE reviews.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>Safety Reviews &amp; PPS Coordination</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D58" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E58" s="11" t="n">
+        <v>174</v>
+      </c>
+      <c r="F58" s="11" t="n">
+        <v>184</v>
+      </c>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H58" s="11" t="inlineStr">
+        <is>
+          <t>PPS review/approval with SLAC AD Safety Division. LOTO procedures, arc flash analysis, OSHA compliance for building/stairway. Formal change control documentation, RSWCF. Early engagement critical (Sec 9.4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr"/>
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>Subtotal WBS 7.0</t>
+        </is>
+      </c>
+      <c r="C59" s="12">
+        <f>SUM(C57:C58)</f>
+        <v/>
+      </c>
+      <c r="D59" s="12" t="n"/>
+      <c r="E59" s="12">
+        <f>SUM(E57:E58)</f>
+        <v/>
+      </c>
+      <c r="F59" s="12">
+        <f>SUM(F57:F58)</f>
+        <v/>
+      </c>
+      <c r="G59" s="12" t="n"/>
+      <c r="H59" s="12" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="B61" s="10" t="inlineStr">
+        <is>
+          <t>INFRASTRUCTURE (Reference - other groups may provide independent estimates)</t>
+        </is>
+      </c>
+      <c r="C61" s="10" t="n"/>
+      <c r="D61" s="10" t="n"/>
+      <c r="E61" s="10" t="n"/>
+      <c r="F61" s="10" t="n"/>
+      <c r="G61" s="10" t="n"/>
+      <c r="H61" s="10" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>480 VAC Distribution System</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="n">
+        <v>900</v>
+      </c>
+      <c r="D62" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E62" s="13" t="n">
+        <v>696</v>
+      </c>
+      <c r="F62" s="13" t="n">
+        <v>1596</v>
+      </c>
+      <c r="G62" s="13" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H62" s="13" t="inlineStr">
+        <is>
+          <t>REFERENCE: Substation 507 option ($1-2M per 1/27 mtg). 2.5-3 MVA transformer 12kV-480V (~$150-200k); 12kV feed + switchgear (~$300k); 480V panels/breakers 4-8 buckets/SSA (~$200k); civil/cable (~$200k). F&amp;O/Andi scope. Alt: Sub 502 = $8-9M.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="13" t="inlineStr">
+        <is>
+          <t>8.2</t>
+        </is>
+      </c>
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>Cooling Water (LCW/HCW)</t>
+        </is>
+      </c>
+      <c r="C63" s="13" t="n">
+        <v>250</v>
+      </c>
+      <c r="D63" s="13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E63" s="13" t="n">
+        <v>522</v>
+      </c>
+      <c r="F63" s="13" t="n">
+        <v>772</v>
+      </c>
+      <c r="G63" s="13" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H63" s="13" t="inlineStr">
+        <is>
+          <t>REFERENCE: 400 GPM LCW for 4 SSA stations. Option B: new 6"+ connection to main header (per 3/10 mtg). 4"-&gt;6"+ piping upgrade ($100-150k); manifolds/valves/controls ($50-75k); HCW for loads ($25-50k). Javier/F&amp;O scope. Summer shutdown required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>8.3</t>
+        </is>
+      </c>
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>Building Extension &amp; Mezzanine</t>
+        </is>
+      </c>
+      <c r="C64" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="D64" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E64" s="13" t="n">
+        <v>696</v>
+      </c>
+      <c r="F64" s="13" t="n">
+        <v>1196</v>
+      </c>
+      <c r="G64" s="13" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H64" s="13" t="inlineStr">
+        <is>
+          <t>REFERENCE: ~636 sqft extension + ~300 sqft mezzanine @ 27 ft. Two-story layout (per 2/24 mtg). OSHA stairway (~25 risers). Roll-up doors. HVAC for SSA heat. Seismic. F&amp;O prior test facility estimate: $1.3M (per 1/27 mtg). Javier/F&amp;O scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr"/>
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>Subtotal WBS 8.0 (Reference)</t>
+        </is>
+      </c>
+      <c r="C65" s="12">
+        <f>SUM(C62:C64)</f>
+        <v/>
+      </c>
+      <c r="D65" s="12" t="n"/>
+      <c r="E65" s="12">
+        <f>SUM(E62:E64)</f>
+        <v/>
+      </c>
+      <c r="F65" s="12">
+        <f>SUM(F62:F64)</f>
+        <v/>
+      </c>
+      <c r="G65" s="12" t="n"/>
+      <c r="H65" s="12" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="inlineStr"/>
+      <c r="B67" s="14" t="inlineStr">
+        <is>
+          <t>RF/CONTROLS SCOPE SUBTOTAL (WBS 1-7)</t>
+        </is>
+      </c>
+      <c r="C67" s="15">
+        <f>C11+C20+C32+C40+C48+C54+C59</f>
+        <v/>
+      </c>
+      <c r="D67" s="14" t="n"/>
+      <c r="E67" s="14">
+        <f>E11+E20+E32+E40+E48+E54+E59</f>
+        <v/>
+      </c>
+      <c r="F67" s="14">
+        <f>F11+F20+F32+F40+F48+F54+F59</f>
+        <v/>
+      </c>
+      <c r="G67" s="14" t="n"/>
+      <c r="H67" s="14" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="n"/>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>INFRASTRUCTURE REFERENCE (WBS 8)</t>
+        </is>
+      </c>
+      <c r="C68" s="14">
+        <f>C65</f>
+        <v/>
+      </c>
+      <c r="D68" s="14" t="n"/>
+      <c r="E68" s="14">
+        <f>E65</f>
+        <v/>
+      </c>
+      <c r="F68" s="14">
+        <f>F65</f>
+        <v/>
+      </c>
+      <c r="G68" s="14" t="n"/>
+      <c r="H68" s="14" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="16" t="n"/>
+      <c r="B69" s="16" t="inlineStr">
+        <is>
+          <t>PROJECT BASE ESTIMATE (WBS 1-8)</t>
+        </is>
+      </c>
+      <c r="C69" s="16">
+        <f>C67+C68</f>
+        <v/>
+      </c>
+      <c r="D69" s="16" t="n"/>
+      <c r="E69" s="16">
+        <f>E67+E68</f>
+        <v/>
+      </c>
+      <c r="F69" s="16">
+        <f>F67+F68</f>
+        <v/>
+      </c>
+      <c r="G69" s="16" t="n"/>
+      <c r="H69" s="16" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr"/>
+      <c r="B71" s="14" t="inlineStr">
+        <is>
+          <t>CONTINGENCY (30% of base, per DOE 413.3B / AACE Class 4)</t>
+        </is>
+      </c>
+      <c r="C71" s="14" t="n"/>
+      <c r="D71" s="14" t="n"/>
+      <c r="E71" s="14" t="n"/>
+      <c r="F71" s="14">
+        <f>F69*0.30</f>
+        <v/>
+      </c>
+      <c r="G71" s="14" t="n"/>
+      <c r="H71" s="14" t="inlineStr">
+        <is>
+          <t>AACE 18R-97 Class 4: typical accuracy range -15% to +30%. DOE Order 413.3B requires contingency at conceptual design. 30% applied to full project base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="16" t="n"/>
+      <c r="B72" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL ESTIMATED COST (Base + Contingency)</t>
+        </is>
+      </c>
+      <c r="C72" s="16" t="n"/>
+      <c r="D72" s="16" t="n"/>
+      <c r="E72" s="16" t="n"/>
+      <c r="F72" s="16">
+        <f>F69+F71</f>
+        <v/>
+      </c>
+      <c r="G72" s="16" t="n"/>
+      <c r="H72" s="16" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="17" t="inlineStr">
+        <is>
+          <t>KEY ASSUMPTIONS &amp; RISKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Electrical based on Substation 507 option. Substation 502 option would add ~$7M to WBS 8.1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Circulator cost assumes new procurement. PEP-II 1.5 MW circulators may be reusable (saves ~$400k in WBS 2.3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>SSA spares (WBS 1.2) assume 2 units. Could be reduced to 1 (saves $312k) or increased per ops requirements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Labor rate: $200/hr burdened (SLAC lab rate including overhead). 1 FTE = 1,740 hrs/yr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>RISK: Interface Chassis on critical path (design not started). PCB iteration may add 3-6 months and $10-20k.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>RISK: Tuner motor controller reliability unproven. May require redesign (adds $20-50k and 0.5 FTE).</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>RISK: EPICS Coordinator software is largest untouched scope. Schedule risk if parallel development insufficient.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>RISK: PPS regulatory approval timeline uncertain. Early engagement with AD Safety Division required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>RISK: DOE lab construction costs typically 50-100% higher than commercial. WBS 8.3 may be significantly understated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>RISK: Limited SPEAR testing windows. Integration testing constrained to summer shutdowns and brief maintenance periods.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B3:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -983,7 +2936,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Fix vendor links & include infrastructure in SSA scope
Vendor link verification (all 36 items checked):
- REMOVED Bird Technologies RF loads: max 20 kW, unsuitable for 250+ kW
  → Replaced with Ferrite Microwave Technologies (FMT) water-cooled loads
- REMOVED SPINNER Group combiners: 8.8 kW broadcast-grade, unsuitable
  → Replaced with Mega Industries (NSLS-II precedent: 4×80kW=320kW @ 500 MHz)
- UPDATED circulators: AFT Microwave unclear at 476 MHz
  → FMT now primary (1400+ designs, WR28-WR2300, 50 MHz-50 GHz)
- All 13 other vendor links verified active and technically appropriate
- Added vendor verification notes section in Reference Pricing

Infrastructure reclassification (per user):
- WBS 8.0 moved from 'Reference (other groups)' to 'Included in SSA scope'
- Updated Class 4 Estimate labels and Project Scope description
- No cost changes — same dollar amounts, now counted as SSA project costs

Co-authored-by: fayaw <faya.wang@gmail.com>
</commit_message>
<xml_diff>
--- a/SSA_upgrade/SSA Upgrade Project Cost V1.xlsx
+++ b/SSA_upgrade/SSA Upgrade Project Cost V1.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -89,6 +89,9 @@
     <font>
       <i val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -162,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="2"/>
@@ -195,6 +198,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -551,6 +555,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="17" t="inlineStr">
         <is>
@@ -579,6 +584,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
@@ -593,6 +599,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
         <is>
@@ -649,6 +656,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
         <is>
@@ -656,6 +664,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="22" t="inlineStr">
         <is>
@@ -684,6 +693,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="22" t="inlineStr">
         <is>
@@ -719,6 +729,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="22" t="inlineStr">
         <is>
@@ -789,6 +800,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" s="22" t="inlineStr">
         <is>
@@ -831,6 +843,7 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
     <row r="51">
       <c r="A51" s="22" t="inlineStr">
         <is>
@@ -873,6 +886,7 @@
         </is>
       </c>
     </row>
+    <row r="57"/>
     <row r="58">
       <c r="A58" s="22" t="inlineStr">
         <is>
@@ -901,6 +915,7 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="A63" s="22" t="inlineStr">
         <is>
@@ -922,17 +937,19 @@
         </is>
       </c>
     </row>
+    <row r="66"/>
     <row r="67">
       <c r="A67" s="17" t="inlineStr">
         <is>
-          <t>4. NOT INCLUDED IN SSA PROJECT SCOPE (reference items or other groups)</t>
-        </is>
-      </c>
-    </row>
+          <t>4. SUPPORTING SCOPE ITEMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="68"/>
     <row r="69">
       <c r="A69" s="22" t="inlineStr">
         <is>
-          <t>4a. Infrastructure (WBS 8.0 - F&amp;O / Facilities scope)</t>
+          <t>4a. Infrastructure (WBS 8.0 - Included in SSA Project)</t>
         </is>
       </c>
     </row>
@@ -960,10 +977,11 @@
     <row r="73">
       <c r="A73" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  These are carried as REFERENCE items for total project budgeting.</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">  These are INCLUDED in the SSA project scope and cost estimate (WBS 8.0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="74"/>
     <row r="75">
       <c r="A75" s="22" t="inlineStr">
         <is>
@@ -1006,6 +1024,7 @@
         </is>
       </c>
     </row>
+    <row r="81"/>
     <row r="82">
       <c r="A82" s="22" t="inlineStr">
         <is>
@@ -1041,6 +1060,7 @@
         </is>
       </c>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="17" t="inlineStr">
         <is>
@@ -1097,6 +1117,7 @@
         </is>
       </c>
     </row>
+    <row r="96"/>
     <row r="97">
       <c r="A97" s="17" t="inlineStr">
         <is>
@@ -1180,7 +1201,7 @@
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
         <is>
-          <t>NOTE: This estimate covers SSA upgrade scope ONLY. LLRF upgrade (klystron/HVPS controls modernization) is a prerequisite project funded separately.</t>
+          <t>NOTE: This estimate covers SSA upgrade scope including infrastructure (WBS 1-8). LLRF upgrade (klystron/HVPS controls modernization) is a prerequisite project funded separately.</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2702,7 @@
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>INFRASTRUCTURE (Reference - F&amp;O / other groups' scope)</t>
+          <t>INFRASTRUCTURE (Included in SSA Project Scope)</t>
         </is>
       </c>
       <c r="C63" s="10" t="n"/>
@@ -2721,7 +2742,7 @@
       </c>
       <c r="H64" s="13" t="inlineStr">
         <is>
-          <t>REF: Sub 507 option ($1-2M per 1/27 mtg). 2.5-3 MVA transformer, 12kV feed, 480V panels for 16 SSAs. Alt: Sub 502 = $8-9M.</t>
+          <t>Sub 507 option ($1-2M per 1/27 mtg). 2.5-3 MVA transformer, 12kV feed, 480V panels for 16 SSAs. Alt: Sub 502 = $8-9M.</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2776,7 @@
       </c>
       <c r="H65" s="13" t="inlineStr">
         <is>
-          <t>REF: 400 GPM LCW for 4 SSA stations. Option B: new 6"+ connection (per 3/10 mtg). Summer shutdown required.</t>
+          <t>400 GPM LCW for 4 SSA stations. Option B: new 6"+ connection (per 3/10 mtg). Summer shutdown required.</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2810,7 @@
       </c>
       <c r="H66" s="13" t="inlineStr">
         <is>
-          <t>REF: ~636 sqft + ~300 sqft mezzanine @ 27 ft. Two-story layout (per 2/24 mtg). OSHA stairway. Roll-up doors. Seismic. F&amp;O prior estimate $1.3M.</t>
+          <t>~636 sqft + ~300 sqft mezzanine @ 27 ft. Two-story layout (per 2/24 mtg). OSHA stairway. Roll-up doors. Seismic. F&amp;O prior estimate $1.3M.</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2818,7 @@
       <c r="A67" s="12" t="inlineStr"/>
       <c r="B67" s="12" t="inlineStr">
         <is>
-          <t>Subtotal WBS 8.0 (Reference)</t>
+          <t>Subtotal WBS 8.0 (Infrastructure)</t>
         </is>
       </c>
       <c r="C67" s="12">
@@ -2843,7 +2864,7 @@
       <c r="A70" s="14" t="n"/>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>INFRASTRUCTURE REFERENCE (WBS 8)</t>
+          <t>INFRASTRUCTURE SCOPE (WBS 8)</t>
         </is>
       </c>
       <c r="C70" s="14">
@@ -3065,7 +3086,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>DOE lab construction costs typically 50-100% higher than commercial. WBS 8.3 may be significantly understated.</t>
+          <t>DOE lab construction costs typically 50-100% higher than commercial. WBS 8.3 building estimate based on F&amp;O prior study ($1.3M); actual cost TBD per CD-1 design.</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3208,22 +3229,22 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>SSA RF Dummy Load (50 kW CW)</t>
+          <t>SSA RF Dummy Load (250 kW CW, water-cooled)</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Bird Technologies / Mega Industries</t>
+          <t>Ferrite Microwave Technologies (FMT)</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>https://www.birdrf.com/Products/RF-Loads.aspx</t>
+          <t>https://ferriteinc.com/high-power-waveguide-terminations/water-cooled-loads/</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Custom WR2100/coax load</t>
+          <t>Custom WR2100 water-cooled load</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -3233,12 +3254,12 @@
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Vendor catalog (verified)</t>
         </is>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>For Bldg 122 test stand; water-cooled</t>
+          <t>FMT: WR28-WR2300 waveguide loads, 50 MHz-50 GHz. MIL-D-3954 compliant. Ultra-high temp refractory ceramic absorber. REPLACES Bird Technologies (max 20 kW, unsuitable).</t>
         </is>
       </c>
     </row>
@@ -3369,22 +3390,22 @@
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>WR2100 Circulator (high power)</t>
+          <t>WR2100 Circulator (250+ kW CW @ 476 MHz)</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Mega Industries / AFT Microwave</t>
+          <t>Ferrite Microwave Technologies (FMT)</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>https://www.megaind.com/products/waveguide-sizes/wr2100-waveguide/</t>
+          <t>https://ferriteinc.com/high-power-microwave-circulators-isolators/waveguide-circulators/</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>WR2100 circulator</t>
+          <t>Custom WR2100 3-port circulator</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -3394,34 +3415,34 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Vendor inquiry (verified)</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Ferrite circulator for 250+ kW CW @ 476 MHz. AFT: aft-microwave.com</t>
+          <t>FMT: 1400+ circulator designs, WR28-WR2300, 50 MHz-50 GHz, 5W to 50+ MW. Scientific/accelerator specialist. AFT Microwave (aft-microwave.com) as alternate (L/S/C/X bands; confirm 476 MHz coverage before ordering).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>WR2100 High Power Load (water-cooled)</t>
+          <t>WR2100 High-Power Water-Cooled Load (circulator termination)</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Mega Industries</t>
+          <t>Ferrite Microwave Technologies (FMT) / MCI Broadcast</t>
         </is>
       </c>
       <c r="C15" s="20" t="inlineStr">
         <is>
-          <t>https://www.megaind.com/products/waveguide-sizes/wr2100-waveguide/</t>
+          <t>https://ferriteinc.com/high-power-waveguide-terminations/water-cooled-loads/</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>WR2100 load</t>
+          <t>WR2100 water load, 250+ kW CW</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
@@ -3431,12 +3452,12 @@
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>Catalog</t>
+          <t>Vendor catalog (verified)</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>Water-cooled dummy load for circulator termination. 250+ kW CW rating.</t>
+          <t>For circulator port 3 termination. FMT water-cooled loads: refractory ceramic absorber, welded aluminum housing. MCI Broadcast (mcibroadcast.com) also makes accelerator-specific waveguide loads 0.32-10 GHz.</t>
         </is>
       </c>
     </row>
@@ -3480,22 +3501,22 @@
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>6-1/8" Coaxial Combiner (4:1)</t>
+          <t>4:1 High-Power Waveguide Combiner (320 kW @ 476 MHz)</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>SPINNER Group / Custom</t>
+          <t>Mega Industries</t>
         </is>
       </c>
       <c r="C17" s="20" t="inlineStr">
         <is>
-          <t>https://products.spinner-group.com/</t>
+          <t>https://www.megaind.com/high-power-waveguide-combiners-for-sspa/</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Custom 4-way combiner</t>
+          <t>Custom WR2100 4:1 combiner (ref: WR1800 NSLS-II design)</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
@@ -3505,12 +3526,12 @@
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Vendor reference (verified)</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>6-1/8" EIA input, WR2100 output. SPINNER makes broadcast combiners; custom for accelerator.</t>
+          <t>PRECEDENT: Mega built WR1800 4:1 combiner for NSLS-II at Brookhaven (500 MHz, 4×80kW=320kW, &lt;0.12 dB loss, &lt;1.18:1 VSWR). Nearly identical to SPEAR3 application (476 MHz, 4×65kW=260kW). REPLACES SPINNER Group (max 8.8 kW broadcast-grade, unsuitable).</t>
         </is>
       </c>
     </row>
@@ -4376,6 +4397,97 @@
       <c r="G44" s="11" t="inlineStr">
         <is>
           <t>Federal standard for electromagnetic radiation exposure limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="22" t="inlineStr">
+        <is>
+          <t>VENDOR VERIFICATION NOTES (March 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="24" t="inlineStr">
+        <is>
+          <t>Bird Technologies</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>REMOVED — Max power 20 kW (8740 Series). Unsuitable for 250+ kW circulator loads. Replaced by FMT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="24" t="inlineStr">
+        <is>
+          <t>SPINNER Group</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>REMOVED — Broadcast-grade combiners (8.8 kW max @ 80.5 MHz). Unsuitable for 260 kW @ 476 MHz. Replaced by Mega Industries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="24" t="inlineStr">
+        <is>
+          <t>AFT Microwave</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>CAUTION — Products focus L/S/C/X bands (GHz range). Confirm 476 MHz coverage before ordering. FMT is preferred.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="24" t="inlineStr">
+        <is>
+          <t>Ferrite Microwave Technologies (FMT)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ADDED — WR28-WR2300, 50 MHz-50 GHz, 1400+ designs. Accelerator specialist. Loads + circulators.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="24" t="inlineStr">
+        <is>
+          <t>Mega Industries SSPA Combiner</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ADDED — NSLS-II precedent: 4×80kW=320kW @ 500 MHz (Brookhaven). Nearly identical to SPEAR3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="24" t="inlineStr">
+        <is>
+          <t>MCI Broadcast</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ADDED — Micro Communications waveguide loads for particle accelerators, 0.32-10 GHz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="24" t="inlineStr">
+        <is>
+          <t>All other vendors</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>VERIFIED — Links confirmed active, components confirmed suitable for 476.3 MHz / WR2100 / high-power CW.</t>
         </is>
       </c>
     </row>

</xml_diff>